<commit_message>
docs: 更新 daily check 历史 2026-06-22
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -405,38 +405,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
         <v>成功</v>
       </c>
       <c r="C1">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D1" t="str">
         <v/>
       </c>
-      <c r="E1">
-        <v>0</v>
+      <c r="E1" t="str">
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/163</v>
       </c>
       <c r="F1">
         <v>0</v>
       </c>
       <c r="G1">
+        <v>0</v>
+      </c>
+      <c r="H1">
         <v>166</v>
       </c>
-      <c r="H1">
+      <c r="I1">
         <v>110</v>
       </c>
-      <c r="I1">
-        <v>2</v>
-      </c>
       <c r="J1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1">
         <v>0</v>
@@ -448,23 +448,26 @@
         <v>0</v>
       </c>
       <c r="N1">
+        <v>0</v>
+      </c>
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
         <v>跳过</v>
@@ -475,8 +478,8 @@
       <c r="D1" t="str">
         <v/>
       </c>
-      <c r="E1">
-        <v>0</v>
+      <c r="E1" t="str">
+        <v/>
       </c>
       <c r="F1">
         <v>0</v>
@@ -503,23 +506,26 @@
         <v>0</v>
       </c>
       <c r="N1">
+        <v>0</v>
+      </c>
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
         <v>成功</v>
@@ -530,8 +536,8 @@
       <c r="D1" t="str">
         <v/>
       </c>
-      <c r="E1">
-        <v>0</v>
+      <c r="E1" t="str">
+        <v/>
       </c>
       <c r="F1">
         <v>0</v>
@@ -558,35 +564,38 @@
         <v>0</v>
       </c>
       <c r="N1">
+        <v>0</v>
+      </c>
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
-        <v>失败</v>
+        <v>成功</v>
       </c>
       <c r="C1">
-        <v>0</v>
+        <v>760</v>
       </c>
       <c r="D1" t="str">
-        <v>spawnSync /bin/sh ETIMEDOUT</v>
-      </c>
-      <c r="E1">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v>https://atomgit.com/opengauss/website/issues/210</v>
       </c>
       <c r="F1">
         <v>0</v>
@@ -595,13 +604,13 @@
         <v>0</v>
       </c>
       <c r="H1">
-        <v>0</v>
+        <v>435</v>
       </c>
       <c r="I1">
-        <v>0</v>
+        <v>313</v>
       </c>
       <c r="J1">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K1">
         <v>0</v>
@@ -613,23 +622,26 @@
         <v>0</v>
       </c>
       <c r="N1">
+        <v>2</v>
+      </c>
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
         <v>成功</v>
@@ -640,8 +652,8 @@
       <c r="D1" t="str">
         <v/>
       </c>
-      <c r="E1">
-        <v>0</v>
+      <c r="E1" t="str">
+        <v/>
       </c>
       <c r="F1">
         <v>0</v>
@@ -668,23 +680,26 @@
         <v>0</v>
       </c>
       <c r="N1">
+        <v>0</v>
+      </c>
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
         <v>跳过</v>
@@ -695,8 +710,8 @@
       <c r="D1" t="str">
         <v/>
       </c>
-      <c r="E1">
-        <v>0</v>
+      <c r="E1" t="str">
+        <v/>
       </c>
       <c r="F1">
         <v>0</v>
@@ -723,23 +738,26 @@
         <v>0</v>
       </c>
       <c r="N1">
+        <v>0</v>
+      </c>
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
         <v>成功</v>
@@ -750,51 +768,54 @@
       <c r="D1" t="str">
         <v/>
       </c>
-      <c r="E1">
-        <v>0</v>
+      <c r="E1" t="str">
+        <v>https://atomgit.com/mindspore/mindspore-portal/issues/96</v>
       </c>
       <c r="F1">
         <v>0</v>
       </c>
       <c r="G1">
+        <v>0</v>
+      </c>
+      <c r="H1">
         <v>1675</v>
       </c>
-      <c r="H1">
+      <c r="I1">
         <v>1714</v>
       </c>
-      <c r="I1">
+      <c r="J1">
         <v>10</v>
       </c>
-      <c r="J1">
-        <v>0</v>
-      </c>
       <c r="K1">
+        <v>0</v>
+      </c>
+      <c r="L1">
         <v>1</v>
       </c>
-      <c r="L1">
-        <v>0</v>
-      </c>
       <c r="M1">
         <v>0</v>
       </c>
       <c r="N1">
+        <v>0</v>
+      </c>
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
         <v>成功</v>
@@ -805,24 +826,24 @@
       <c r="D1" t="str">
         <v/>
       </c>
-      <c r="E1">
-        <v>0</v>
+      <c r="E1" t="str">
+        <v>https://atomgit.com/openUBMC/website/issues/85</v>
       </c>
       <c r="F1">
         <v>0</v>
       </c>
       <c r="G1">
+        <v>0</v>
+      </c>
+      <c r="H1">
         <v>59</v>
       </c>
-      <c r="H1">
+      <c r="I1">
         <v>62</v>
       </c>
-      <c r="I1">
+      <c r="J1">
         <v>10</v>
       </c>
-      <c r="J1">
-        <v>0</v>
-      </c>
       <c r="K1">
         <v>0</v>
       </c>
@@ -830,54 +851,57 @@
         <v>0</v>
       </c>
       <c r="M1">
+        <v>0</v>
+      </c>
+      <c r="N1">
         <v>1</v>
       </c>
-      <c r="N1">
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>2026-06-22 07:38:51</v>
+        <v>2026-06-22 08:47:48</v>
       </c>
       <c r="B1" t="str">
         <v>成功</v>
       </c>
       <c r="C1">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D1" t="str">
         <v/>
       </c>
-      <c r="E1">
-        <v>0</v>
+      <c r="E1" t="str">
+        <v/>
       </c>
       <c r="F1">
         <v>0</v>
       </c>
       <c r="G1">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H1">
         <v>27</v>
       </c>
       <c r="I1">
+        <v>27</v>
+      </c>
+      <c r="J1">
         <v>10</v>
       </c>
-      <c r="J1">
-        <v>0</v>
-      </c>
       <c r="K1">
         <v>0</v>
       </c>
@@ -885,15 +909,18 @@
         <v>0</v>
       </c>
       <c r="M1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N1">
+        <v>2</v>
+      </c>
+      <c r="O1">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-06-23
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -483,7 +483,7 @@
         <v>110</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -771,13 +771,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -810,7 +810,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -876,7 +876,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1086,7 +1086,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1191,7 +1191,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1296,13 +1296,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-22 09:57:52</v>
+        <v>2026-06-23 06:28:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1335,7 +1335,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-06-24
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -483,7 +483,7 @@
         <v>110</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -771,7 +771,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -876,7 +876,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1086,7 +1086,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1191,7 +1191,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1212,10 +1212,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J2">
         <v>10</v>
@@ -1296,13 +1296,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-23 06:28:09</v>
+        <v>2026-06-24 06:28:20</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1335,7 +1335,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-06-25
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -483,7 +483,7 @@
         <v>110</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -771,7 +771,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -876,7 +876,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1086,13 +1086,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>3400</v>
+        <v>3401</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1116,7 +1116,7 @@
         <v>10</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2">
         <v>1</v>
@@ -1191,7 +1191,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1296,7 +1296,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-24 06:28:20</v>
+        <v>2026-06-25 06:27:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-06-26
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -771,20 +771,20 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-26 07:27:43</v>
       </c>
       <c r="B2" t="str">
-        <v>成功</v>
+        <v>失败</v>
       </c>
       <c r="C2">
-        <v>759</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
+        <v>ENOENT: no such file or directory, open '/tmp/.cache/geo-bot/semantic-check/render-input-openGauss-1782458863766.txt'</v>
+      </c>
+      <c r="E2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/opengauss/website/issues/210</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
@@ -792,13 +792,13 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>435</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>313</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -810,7 +810,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-06-27
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>277</v>
+        <v>5</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -477,25 +477,25 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>166</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
         <v>1</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -666,19 +666,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>https://atomgit.com/openeuler/docs-website/issues/34</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -705,7 +705,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -771,13 +771,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-26 08:54:33</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>790</v>
+        <v>784</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -810,10 +810,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -876,19 +876,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>https://atomgit.com/opengauss/docs-website/issues/12</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -915,7 +915,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1086,20 +1086,20 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
-        <v>成功</v>
+        <v>失败</v>
       </c>
       <c r="C2">
-        <v>3401</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
+        <v>Maximum call stack size exceeded</v>
+      </c>
+      <c r="E2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/mindspore/mindspore-portal/issues/96</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
@@ -1107,19 +1107,19 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>1675</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>1714</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -1191,13 +1191,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>132</v>
+        <v>279</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1221,7 +1221,7 @@
         <v>10</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1233,7 +1233,7 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1296,13 +1296,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-25 06:27:31</v>
+        <v>2026-06-27 06:35:47</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1326,7 +1326,7 @@
         <v>10</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1335,7 +1335,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-06-28
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -771,13 +771,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -810,10 +810,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O2">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -876,7 +876,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1086,7 +1086,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1191,13 +1191,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1212,16 +1212,16 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1230,10 +1230,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1296,13 +1296,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-27 06:35:47</v>
+        <v>2026-06-28 07:02:33</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D2" t="str">
         <v/>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-06-29
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-28 07:02:33</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -483,7 +483,7 @@
         <v>2</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -561,7 +561,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-28 07:02:33</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-28 07:02:33</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -771,13 +771,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-28 07:02:33</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>785</v>
+        <v>801</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -876,7 +876,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-28 07:02:33</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-28 07:02:33</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1086,7 +1086,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 02:18:05</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1191,13 +1191,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-28 07:02:33</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1230,7 +1230,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1296,13 +1296,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-28 07:02:33</v>
+        <v>2026-06-29 07:24:31</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1335,7 +1335,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-01
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -498,7 +498,7 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -561,7 +561,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -771,13 +771,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>801</v>
+        <v>782</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -810,10 +810,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -876,7 +876,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1086,19 +1086,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
-        <v>失败</v>
+        <v>成功</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3412</v>
       </c>
       <c r="D2" t="str">
-        <v>Maximum call stack size exceeded</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>https://atomgit.com/mindspore/mindspore-portal/issues/96</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1107,19 +1107,19 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>1675</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1713</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -1128,7 +1128,7 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1191,19 +1191,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>https://atomgit.com/openUBMC/website/issues/85</v>
+        <v/>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1221,7 +1221,7 @@
         <v>10</v>
       </c>
       <c r="K2">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1230,7 +1230,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1296,13 +1296,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-06-29 07:24:31</v>
+        <v>2026-07-01 07:18:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1335,7 +1335,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-02
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 07:18:06</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -483,7 +483,7 @@
         <v>2</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -498,7 +498,7 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -561,7 +561,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 07:18:06</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 07:18:06</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -771,13 +771,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 09:27:28</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>788</v>
+        <v>764</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -813,7 +813,7 @@
         <v>3</v>
       </c>
       <c r="O2">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -876,7 +876,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 07:18:06</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 07:18:06</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1086,7 +1086,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 07:18:06</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1128,7 +1128,7 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1191,13 +1191,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 07:18:06</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1230,7 +1230,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1296,7 +1296,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-01 07:18:06</v>
+        <v>2026-07-02 06:51:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-03
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -720,7 +720,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -769,21 +769,29 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-02 16:12:58</v>
+        <v>2026-07-03 07:28:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/opengauss/website/issues/245</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/248
+https://atomgit.com/opengauss/website/issues/249
+https://atomgit.com/opengauss/website/issues/250
+https://atomgit.com/opengauss/website/issues/251
+https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/253
+https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/255
+https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -813,12 +821,15 @@
         <v>4</v>
       </c>
       <c r="O2">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="P2">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-04
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,21 +454,28 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-02 06:51:38</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/163</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
+https://atomgit.com/openeuler/openEuler-portal/issues/185
+https://atomgit.com/openeuler/openEuler-portal/issues/186
+https://atomgit.com/openeuler/openEuler-portal/issues/187
+https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/189
+https://atomgit.com/openeuler/openEuler-portal/issues/190
+https://atomgit.com/openeuler/openEuler-portal/issues/191</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -483,34 +490,37 @@
         <v>2</v>
       </c>
       <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
         <v>2</v>
       </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
       <c r="O2">
-        <v>9</v>
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -561,7 +571,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-03 02:44:46</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -605,17 +615,20 @@
       <c r="O2">
         <v>0</v>
       </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -666,7 +679,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-02 06:51:38</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -678,7 +691,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/docs-website/issues/34</v>
+        <v>https://atomgit.com/openeuler/docs-website/issues/37</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -710,10 +723,13 @@
       <c r="O2">
         <v>0</v>
       </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -771,13 +787,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-03 09:48:17</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -789,9 +805,9 @@
 https://atomgit.com/opengauss/website/issues/251
 https://atomgit.com/opengauss/website/issues/252
 https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/257
-https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/258</v>
+https://atomgit.com/opengauss/website/issues/255
+https://atomgit.com/opengauss/website/issues/258
+https://atomgit.com/opengauss/website/issues/254</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -818,13 +834,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -836,7 +852,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -887,7 +903,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-02 06:51:38</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -899,7 +915,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>https://atomgit.com/opengauss/docs-website/issues/12</v>
+        <v>https://atomgit.com/opengauss/docs-website/issues/14</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -931,17 +947,20 @@
       <c r="O2">
         <v>0</v>
       </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -992,7 +1011,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-02 06:51:38</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1036,17 +1055,20 @@
       <c r="O2">
         <v>0</v>
       </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1095,21 +1117,35 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-02 06:51:38</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>3412</v>
+        <v>3403</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/mindspore/mindspore-portal/issues/96</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
+https://atomgit.com/mindspore/mindspore-portal/issues/128
+https://atomgit.com/mindspore/mindspore-portal/issues/129
+https://atomgit.com/mindspore/mindspore-portal/issues/130
+https://atomgit.com/mindspore/mindspore-portal/issues/131
+https://atomgit.com/mindspore/mindspore-portal/issues/132
+https://atomgit.com/mindspore/mindspore-portal/issues/133
+https://atomgit.com/mindspore/mindspore-portal/issues/134
+https://atomgit.com/mindspore/mindspore-portal/issues/135
+https://atomgit.com/mindspore/mindspore-portal/issues/136
+https://atomgit.com/mindspore/mindspore-portal/issues/137
+https://atomgit.com/mindspore/mindspore-portal/issues/138
+https://atomgit.com/mindspore/mindspore-portal/issues/139
+https://atomgit.com/mindspore/mindspore-portal/issues/140
+https://atomgit.com/mindspore/mindspore-portal/issues/141</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1141,17 +1177,20 @@
       <c r="O2">
         <v>0</v>
       </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1202,7 +1241,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-02 06:51:38</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1223,16 +1262,16 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1246,17 +1285,20 @@
       <c r="O2">
         <v>0</v>
       </c>
+      <c r="P2">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1307,7 +1349,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-02 06:51:38</v>
+        <v>2026-07-04 06:23:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1351,10 +1393,13 @@
       <c r="O2">
         <v>0</v>
       </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-05
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -471,11 +471,7 @@
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/186
-https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/191</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -508,7 +504,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +567,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -679,7 +675,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -787,13 +783,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -804,10 +800,7 @@
 https://atomgit.com/opengauss/website/issues/250
 https://atomgit.com/opengauss/website/issues/251
 https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/255
-https://atomgit.com/opengauss/website/issues/258
-https://atomgit.com/opengauss/website/issues/254</v>
+https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -834,13 +827,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P2">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -903,7 +896,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1011,7 +1004,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1119,7 +1112,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1241,13 +1234,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1286,7 +1279,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1349,13 +1342,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-04 06:23:37</v>
+        <v>2026-07-05 06:37:42</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1388,13 +1381,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-06
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -471,7 +471,14 @@
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/186
-https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187
+https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/191
+https://atomgit.com/openeuler/openEuler-portal/issues/189
+https://atomgit.com/openeuler/openEuler-portal/issues/192
+https://atomgit.com/openeuler/openEuler-portal/issues/190
+https://atomgit.com/openeuler/openEuler-portal/issues/193
+https://atomgit.com/openeuler/openEuler-portal/issues/194</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -498,13 +505,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -567,7 +574,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -675,7 +682,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -783,13 +790,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -800,7 +807,9 @@
 https://atomgit.com/opengauss/website/issues/250
 https://atomgit.com/opengauss/website/issues/251
 https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/256</v>
+https://atomgit.com/opengauss/website/issues/253
+https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/258</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -827,13 +836,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -896,7 +905,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1004,7 +1013,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1112,7 +1121,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1234,13 +1243,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1279,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1342,13 +1351,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-05 06:37:42</v>
+        <v>2026-07-06 07:15:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1381,13 +1390,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-07
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -788,28 +788,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-07 03:09:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/248
-https://atomgit.com/opengauss/website/issues/249
-https://atomgit.com/opengauss/website/issues/250
-https://atomgit.com/opengauss/website/issues/251
-https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/258</v>
+      <c r="E2" t="str">
+        <v/>
       </c>
       <c r="F2">
         <v>0</v>
@@ -818,10 +811,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J2">
         <v>10</v>
@@ -836,13 +829,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-08
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -473,11 +473,10 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/186
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/191
-https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/192
 https://atomgit.com/openeuler/openEuler-portal/issues/190
 https://atomgit.com/openeuler/openEuler-portal/issues/193
+https://atomgit.com/openeuler/openEuler-portal/issues/189
+https://atomgit.com/openeuler/openEuler-portal/issues/202
 https://atomgit.com/openeuler/openEuler-portal/issues/194</v>
       </c>
       <c r="F2">
@@ -493,7 +492,7 @@
         <v>2</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -508,10 +507,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="P2">
-        <v>43</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -574,7 +573,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -682,7 +681,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -788,21 +787,30 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-07 06:41:18</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v/>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
+https://atomgit.com/opengauss/website/issues/248
+https://atomgit.com/opengauss/website/issues/250
+https://atomgit.com/opengauss/website/issues/251
+https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/253
+https://atomgit.com/opengauss/website/issues/257
+https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/255
+https://atomgit.com/opengauss/website/issues/258</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -835,7 +843,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -898,7 +906,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1006,7 +1014,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1114,33 +1122,24 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>3403</v>
+        <v>86</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
-https://atomgit.com/mindspore/mindspore-portal/issues/128
-https://atomgit.com/mindspore/mindspore-portal/issues/129
-https://atomgit.com/mindspore/mindspore-portal/issues/130
-https://atomgit.com/mindspore/mindspore-portal/issues/131
-https://atomgit.com/mindspore/mindspore-portal/issues/132
 https://atomgit.com/mindspore/mindspore-portal/issues/133
-https://atomgit.com/mindspore/mindspore-portal/issues/134
-https://atomgit.com/mindspore/mindspore-portal/issues/135
-https://atomgit.com/mindspore/mindspore-portal/issues/136
-https://atomgit.com/mindspore/mindspore-portal/issues/137
-https://atomgit.com/mindspore/mindspore-portal/issues/138
-https://atomgit.com/mindspore/mindspore-portal/issues/139
 https://atomgit.com/mindspore/mindspore-portal/issues/140
-https://atomgit.com/mindspore/mindspore-portal/issues/141</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/142
+https://atomgit.com/mindspore/mindspore-portal/issues/143
+https://atomgit.com/mindspore/mindspore-portal/issues/149</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1149,19 +1148,19 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>1675</v>
+        <v>21</v>
       </c>
       <c r="I2">
-        <v>1713</v>
+        <v>57</v>
       </c>
       <c r="J2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>4</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -1173,7 +1172,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1236,13 +1235,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1281,7 +1280,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1344,13 +1343,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-06 07:15:23</v>
+        <v>2026-07-08 06:05:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1383,13 +1382,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-09
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -472,12 +472,11 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/186
 https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/188
 https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/193
 https://atomgit.com/openeuler/openEuler-portal/issues/189
 https://atomgit.com/openeuler/openEuler-portal/issues/202
-https://atomgit.com/openeuler/openEuler-portal/issues/194</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/191</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -492,7 +491,7 @@
         <v>2</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -507,10 +506,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -573,7 +572,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -681,7 +680,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -789,13 +788,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -807,10 +806,9 @@
 https://atomgit.com/opengauss/website/issues/251
 https://atomgit.com/opengauss/website/issues/252
 https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/257
 https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/255
-https://atomgit.com/opengauss/website/issues/258</v>
+https://atomgit.com/opengauss/website/issues/258
+https://atomgit.com/opengauss/website/issues/257</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -819,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="I2">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="J2">
         <v>10</v>
@@ -843,7 +841,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -906,7 +904,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1014,7 +1012,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1122,13 +1120,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1136,10 +1134,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
-https://atomgit.com/mindspore/mindspore-portal/issues/140
-https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/149</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/140</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1172,7 +1167,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1235,13 +1230,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1280,7 +1275,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1343,13 +1338,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-08 06:05:07</v>
+        <v>2026-07-09 06:45:37</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1388,7 +1383,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-10
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,13 +470,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/186
 https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/202
-https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/191</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/194</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -491,7 +486,7 @@
         <v>2</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -506,10 +501,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P2">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -572,7 +567,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -680,7 +675,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -788,13 +783,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -802,13 +797,11 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
 https://atomgit.com/opengauss/website/issues/248
-https://atomgit.com/opengauss/website/issues/250
-https://atomgit.com/opengauss/website/issues/251
 https://atomgit.com/opengauss/website/issues/252
 https://atomgit.com/opengauss/website/issues/253
 https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/258
-https://atomgit.com/opengauss/website/issues/257</v>
+https://atomgit.com/opengauss/website/issues/255
+https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -817,31 +810,31 @@
         <v>0</v>
       </c>
       <c r="H2">
+        <v>9</v>
+      </c>
+      <c r="I2">
+        <v>12</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>4</v>
+      </c>
+      <c r="O2">
+        <v>6</v>
+      </c>
+      <c r="P2">
         <v>10</v>
-      </c>
-      <c r="I2">
-        <v>13</v>
-      </c>
-      <c r="J2">
-        <v>10</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>3</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -904,7 +897,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1012,7 +1005,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1120,13 +1113,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1134,7 +1127,11 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
-https://atomgit.com/mindspore/mindspore-portal/issues/140</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/140
+https://atomgit.com/mindspore/mindspore-portal/issues/142
+https://atomgit.com/mindspore/mindspore-portal/issues/143
+https://atomgit.com/mindspore/mindspore-portal/issues/149
+https://atomgit.com/mindspore/mindspore-portal/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1146,7 +1143,7 @@
         <v>21</v>
       </c>
       <c r="I2">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -1164,10 +1161,10 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1230,13 +1227,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1251,16 +1248,16 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I2">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1269,13 +1266,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1338,13 +1335,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-09 06:45:37</v>
+        <v>2026-07-10 06:58:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1377,13 +1374,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-11
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>14</v>
+        <v>145</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -480,10 +480,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -501,7 +501,7 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -783,13 +783,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -797,11 +797,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
 https://atomgit.com/opengauss/website/issues/248
-https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/255
-https://atomgit.com/opengauss/website/issues/256</v>
+https://atomgit.com/opengauss/website/issues/252</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -828,13 +824,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +893,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1005,7 +1001,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1113,13 +1109,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1129,9 +1125,7 @@
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
 https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/149
-https://atomgit.com/mindspore/mindspore-portal/issues/153</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/143</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1161,10 +1155,10 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1227,13 +1221,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1266,13 +1260,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1335,13 +1329,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-10 06:58:04</v>
+        <v>2026-07-11 06:03:18</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1374,13 +1368,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-12
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>145</v>
+        <v>89</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,8 +470,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/194</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -501,7 +500,7 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -567,7 +566,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -675,7 +674,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -783,13 +782,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -824,7 +823,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -893,7 +892,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1001,7 +1000,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1109,13 +1108,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1125,7 +1124,11 @@
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
 https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/143</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/147
+https://atomgit.com/mindspore/mindspore-portal/issues/145
+https://atomgit.com/mindspore/mindspore-portal/issues/143
+https://atomgit.com/mindspore/mindspore-portal/issues/148
+https://atomgit.com/mindspore/mindspore-portal/issues/144</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1158,7 +1161,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1221,13 +1224,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1260,13 +1263,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1329,13 +1332,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-11 06:03:18</v>
+        <v>2026-07-12 06:08:11</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1368,13 +1371,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-13
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>89</v>
+        <v>126</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,7 +470,13 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187
+https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/207
+https://atomgit.com/openeuler/openEuler-portal/issues/190
+https://atomgit.com/openeuler/openEuler-portal/issues/191
+https://atomgit.com/openeuler/openEuler-portal/issues/193
+https://atomgit.com/openeuler/openEuler-portal/issues/202</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -503,7 +509,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -566,7 +572,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -674,7 +680,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -782,13 +788,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -796,7 +802,12 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
 https://atomgit.com/opengauss/website/issues/248
-https://atomgit.com/opengauss/website/issues/252</v>
+https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/253
+https://atomgit.com/opengauss/website/issues/255
+https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/258
+https://atomgit.com/opengauss/website/issues/265</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -823,13 +834,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -892,7 +903,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1000,7 +1011,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1108,13 +1119,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1123,12 +1134,11 @@
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
+https://atomgit.com/mindspore/mindspore-portal/issues/154
 https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/147
-https://atomgit.com/mindspore/mindspore-portal/issues/145
 https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/148
-https://atomgit.com/mindspore/mindspore-portal/issues/144</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/149
+https://atomgit.com/mindspore/mindspore-portal/issues/148</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1161,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1224,13 +1234,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1269,7 +1279,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1332,13 +1342,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-12 06:08:11</v>
+        <v>2026-07-13 06:17:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1371,13 +1381,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-14
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>126</v>
+        <v>89</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,13 +470,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/207
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/191
-https://atomgit.com/openeuler/openEuler-portal/issues/193
-https://atomgit.com/openeuler/openEuler-portal/issues/202</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -509,7 +503,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>37</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -572,7 +566,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -680,7 +674,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -788,13 +782,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -804,10 +798,13 @@
 https://atomgit.com/opengauss/website/issues/248
 https://atomgit.com/opengauss/website/issues/252
 https://atomgit.com/opengauss/website/issues/253
+https://atomgit.com/opengauss/website/issues/266
+https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/257
+https://atomgit.com/opengauss/website/issues/258
 https://atomgit.com/opengauss/website/issues/255
-https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/258
-https://atomgit.com/opengauss/website/issues/265</v>
+https://atomgit.com/opengauss/website/issues/265
+https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -834,13 +831,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P2">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -903,7 +900,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1011,7 +1008,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1119,13 +1116,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1134,11 +1131,9 @@
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
-https://atomgit.com/mindspore/mindspore-portal/issues/154
 https://atomgit.com/mindspore/mindspore-portal/issues/142
 https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/149
-https://atomgit.com/mindspore/mindspore-portal/issues/148</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/149</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1171,7 +1166,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1234,13 +1229,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>286</v>
+        <v>307</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1255,16 +1250,16 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1279,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1342,13 +1337,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-13 06:17:23</v>
+        <v>2026-07-14 05:31:14</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1381,13 +1376,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-15
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,7 +470,11 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187
+https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/190
+https://atomgit.com/openeuler/openEuler-portal/issues/189
+https://atomgit.com/openeuler/openEuler-portal/issues/202</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -503,7 +507,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -566,7 +570,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -674,7 +678,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -782,13 +786,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -798,13 +802,8 @@
 https://atomgit.com/opengauss/website/issues/248
 https://atomgit.com/opengauss/website/issues/252
 https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/266
 https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/257
-https://atomgit.com/opengauss/website/issues/258
-https://atomgit.com/opengauss/website/issues/255
-https://atomgit.com/opengauss/website/issues/265
-https://atomgit.com/opengauss/website/issues/256</v>
+https://atomgit.com/opengauss/website/issues/257</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -831,13 +830,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O2">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -900,7 +899,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1008,7 +1007,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1116,13 +1115,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1131,9 +1130,10 @@
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
+https://atomgit.com/mindspore/mindspore-portal/issues/143
 https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/149</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/149
+https://atomgit.com/mindspore/mindspore-portal/issues/147</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1166,7 +1166,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1229,13 +1229,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>307</v>
+        <v>288</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1268,13 +1268,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1337,13 +1337,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-14 05:31:14</v>
+        <v>2026-07-15 05:28:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1376,13 +1376,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-16
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -471,10 +471,7 @@
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/202</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/194</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -504,10 +501,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +567,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -678,7 +675,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -786,13 +783,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -801,9 +798,9 @@
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
 https://atomgit.com/opengauss/website/issues/248
 https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/257
 https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/257</v>
+https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -830,13 +827,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P2">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -899,7 +896,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1007,7 +1004,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1115,13 +1112,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1129,11 +1126,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
-https://atomgit.com/mindspore/mindspore-portal/issues/140
-https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/149
-https://atomgit.com/mindspore/mindspore-portal/issues/147</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/140</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1166,7 +1159,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1229,13 +1222,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>288</v>
+        <v>305</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1250,16 +1243,16 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I2">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J2">
         <v>10</v>
       </c>
       <c r="K2">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1268,13 +1261,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1337,13 +1330,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-15 05:28:23</v>
+        <v>2026-07-16 05:47:06</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1382,7 +1375,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-17
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -471,7 +471,11 @@
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/194</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/190
+https://atomgit.com/openeuler/openEuler-portal/issues/191
+https://atomgit.com/openeuler/openEuler-portal/issues/189
+https://atomgit.com/openeuler/openEuler-portal/issues/202</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -501,10 +505,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -567,7 +571,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -675,7 +679,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -783,13 +787,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -798,8 +802,10 @@
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
 https://atomgit.com/opengauss/website/issues/248
 https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/257
-https://atomgit.com/opengauss/website/issues/253
+https://atomgit.com/opengauss/website/issues/266
+https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/255
+https://atomgit.com/opengauss/website/issues/258
 https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
@@ -827,13 +833,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O2">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -896,7 +902,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1004,7 +1010,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1112,13 +1118,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1126,7 +1132,10 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
-https://atomgit.com/mindspore/mindspore-portal/issues/140</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/140
+https://atomgit.com/mindspore/mindspore-portal/issues/142
+https://atomgit.com/mindspore/mindspore-portal/issues/143
+https://atomgit.com/mindspore/mindspore-portal/issues/149</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1159,7 +1168,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1222,13 +1231,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1261,13 +1270,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1330,13 +1339,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-16 05:47:06</v>
+        <v>2026-07-17 05:53:40</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1369,13 +1378,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-18
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -472,10 +472,9 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/202
 https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/191
-https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/202</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/189</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -508,7 +507,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +570,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -679,7 +678,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -787,13 +786,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -801,12 +800,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
 https://atomgit.com/opengauss/website/issues/248
-https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/266
-https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/255
-https://atomgit.com/opengauss/website/issues/258
-https://atomgit.com/opengauss/website/issues/256</v>
+https://atomgit.com/opengauss/website/issues/252</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -833,13 +827,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -902,7 +896,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1010,7 +1004,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1118,7 +1112,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1135,7 +1129,7 @@
 https://atomgit.com/mindspore/mindspore-portal/issues/140
 https://atomgit.com/mindspore/mindspore-portal/issues/142
 https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/149</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/145</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1231,13 +1225,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1276,7 +1270,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1339,13 +1333,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-17 05:53:40</v>
+        <v>2026-07-18 05:21:12</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1384,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-19
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -472,9 +472,8 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/202
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/189</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/189
+https://atomgit.com/openeuler/openEuler-portal/issues/190</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -507,7 +506,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +569,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -678,7 +677,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -786,13 +785,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -827,7 +826,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -896,7 +895,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1004,7 +1003,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1112,13 +1111,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1128,8 +1127,12 @@
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
 https://atomgit.com/mindspore/mindspore-portal/issues/142
+https://atomgit.com/mindspore/mindspore-portal/issues/155
+https://atomgit.com/mindspore/mindspore-portal/issues/149
+https://atomgit.com/mindspore/mindspore-portal/issues/156
+https://atomgit.com/mindspore/mindspore-portal/issues/144
 https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/145</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/157</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1162,7 +1165,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1225,13 +1228,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1270,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1333,13 +1336,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-18 05:21:12</v>
+        <v>2026-07-19 05:59:07</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1372,13 +1375,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-20
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -472,8 +472,10 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/191
+https://atomgit.com/openeuler/openEuler-portal/issues/190
 https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/190</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/192</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -506,7 +508,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -569,7 +571,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -677,7 +679,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -785,13 +787,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -799,7 +801,8 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
 https://atomgit.com/opengauss/website/issues/248
-https://atomgit.com/opengauss/website/issues/252</v>
+https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -826,10 +829,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -895,7 +898,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1003,7 +1006,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1111,13 +1114,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1127,12 +1130,9 @@
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
 https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/155
-https://atomgit.com/mindspore/mindspore-portal/issues/149
-https://atomgit.com/mindspore/mindspore-portal/issues/156
-https://atomgit.com/mindspore/mindspore-portal/issues/144
+https://atomgit.com/mindspore/mindspore-portal/issues/147
 https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/157</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/149</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1165,7 +1165,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1228,13 +1228,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1267,13 +1267,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1336,7 +1336,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-19 05:59:07</v>
+        <v>2026-07-20 06:19:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-21
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -472,10 +472,7 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/191
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/192</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/190</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -508,7 +505,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +568,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -679,7 +676,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -787,21 +784,19 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/249
-https://atomgit.com/opengauss/website/issues/248
-https://atomgit.com/opengauss/website/issues/252
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
 https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
@@ -811,10 +806,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -829,10 +824,10 @@
         <v>0</v>
       </c>
       <c r="N2">
+        <v>3</v>
+      </c>
+      <c r="O2">
         <v>2</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -898,7 +893,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1006,7 +1001,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1114,13 +1109,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1129,10 +1124,8 @@
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
-https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/147
-https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/149</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/158
+https://atomgit.com/mindspore/mindspore-portal/issues/144</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1165,7 +1158,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1228,13 +1221,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1267,13 +1260,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1336,13 +1329,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-20 06:19:09</v>
+        <v>2026-07-21 05:58:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1375,13 +1368,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-22
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -472,7 +472,9 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/190</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/190
+https://atomgit.com/openeuler/openEuler-portal/issues/202
+https://atomgit.com/openeuler/openEuler-portal/issues/189</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -505,7 +507,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -568,7 +570,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -676,7 +678,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -784,20 +786,23 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/256</v>
+https://atomgit.com/opengauss/website/issues/253
+https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/257
+https://atomgit.com/opengauss/website/issues/258</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -824,13 +829,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -893,7 +898,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1001,7 +1006,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1109,13 +1114,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1124,8 +1129,10 @@
         <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
 https://atomgit.com/mindspore/mindspore-portal/issues/133
 https://atomgit.com/mindspore/mindspore-portal/issues/140
-https://atomgit.com/mindspore/mindspore-portal/issues/158
-https://atomgit.com/mindspore/mindspore-portal/issues/144</v>
+https://atomgit.com/mindspore/mindspore-portal/issues/142
+https://atomgit.com/mindspore/mindspore-portal/issues/143
+https://atomgit.com/mindspore/mindspore-portal/issues/149
+https://atomgit.com/mindspore/mindspore-portal/issues/145</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1158,7 +1165,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1221,13 +1228,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>293</v>
+        <v>16</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1242,16 +1249,16 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>146</v>
+        <v>0</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1266,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1329,13 +1336,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-21 05:58:09</v>
+        <v>2026-07-22 05:56:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1374,7 +1381,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-23
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,25 +456,27 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>99</v>
+        <v>292</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/184
-https://atomgit.com/openeuler/openEuler-portal/issues/185
+        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/189
 https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/202
-https://atomgit.com/openeuler/openEuler-portal/issues/189</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/191
+https://atomgit.com/openeuler/openEuler-portal/issues/215
+https://atomgit.com/openeuler/openEuler-portal/issues/216
+https://atomgit.com/openeuler/openEuler-portal/issues/202</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -483,10 +485,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>44</v>
+        <v>260</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -507,7 +509,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>10</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +572,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -678,7 +680,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -784,25 +786,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/257
-https://atomgit.com/opengauss/website/issues/258</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/opengauss/website/issues/252</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -829,13 +827,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -898,7 +896,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1006,7 +1004,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1112,28 +1110,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
-        <v>成功</v>
+        <v>失败</v>
       </c>
       <c r="C2">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
+        <v>Cannot create property 'border-width' on string 'inherit'</v>
+      </c>
+      <c r="E2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/mindspore/mindspore-portal/issues/127
-https://atomgit.com/mindspore/mindspore-portal/issues/133
-https://atomgit.com/mindspore/mindspore-portal/issues/140
-https://atomgit.com/mindspore/mindspore-portal/issues/142
-https://atomgit.com/mindspore/mindspore-portal/issues/143
-https://atomgit.com/mindspore/mindspore-portal/issues/149
-https://atomgit.com/mindspore/mindspore-portal/issues/145</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
@@ -1141,16 +1133,16 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1165,7 +1157,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1228,13 +1220,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1273,7 +1265,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1336,13 +1328,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-22 05:56:32</v>
+        <v>2026-07-23 06:04:04</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1357,10 +1349,10 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="I2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J2">
         <v>10</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-24
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>292</v>
+        <v>342</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,13 +470,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/191
-https://atomgit.com/openeuler/openEuler-portal/issues/215
-https://atomgit.com/openeuler/openEuler-portal/issues/216
-https://atomgit.com/openeuler/openEuler-portal/issues/202</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/217</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -506,10 +500,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="P2">
-        <v>31</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -572,7 +566,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -680,7 +674,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -788,13 +782,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -827,7 +821,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -896,7 +890,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1004,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1112,7 +1106,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1220,13 +1214,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1265,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1328,13 +1322,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-23 06:04:04</v>
+        <v>2026-07-24 06:07:38</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1373,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-25
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>342</v>
+        <v>273</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,6 +470,10 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
+https://atomgit.com/openeuler/openEuler-portal/issues/189
+https://atomgit.com/openeuler/openEuler-portal/issues/190
+https://atomgit.com/openeuler/openEuler-portal/issues/219
+https://atomgit.com/openeuler/openEuler-portal/issues/191
 https://atomgit.com/openeuler/openEuler-portal/issues/217</v>
       </c>
       <c r="F2">
@@ -500,10 +504,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>81</v>
+        <v>4</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -566,7 +570,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -674,7 +678,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -780,21 +784,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/opengauss/website/issues/252</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/256</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -824,7 +829,7 @@
         <v>2</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -890,7 +895,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -998,7 +1003,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1106,7 +1111,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1214,13 +1219,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1259,7 +1264,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1322,13 +1327,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-24 06:07:38</v>
+        <v>2026-07-25 05:58:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1367,7 +1372,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-26
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,25 +456,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/189
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/219
-https://atomgit.com/openeuler/openEuler-portal/issues/191
-https://atomgit.com/openeuler/openEuler-portal/issues/217</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -504,10 +499,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -678,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -786,20 +781,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/256</v>
+https://atomgit.com/opengauss/website/issues/257
+https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/255</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -826,13 +823,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +892,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1003,7 +1000,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1111,7 +1108,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1219,13 +1216,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1264,7 +1261,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1327,13 +1324,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-25 05:58:05</v>
+        <v>2026-07-26 06:08:23</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1366,13 +1363,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-27
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,20 +456,24 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>261</v>
+        <v>275</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187
+https://atomgit.com/openeuler/openEuler-portal/issues/188
+https://atomgit.com/openeuler/openEuler-portal/issues/190
+https://atomgit.com/openeuler/openEuler-portal/issues/219
+https://atomgit.com/openeuler/openEuler-portal/issues/191</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -502,7 +506,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -565,7 +569,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +677,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -781,21 +785,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/257
+https://atomgit.com/opengauss/website/issues/253
 https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/266
 https://atomgit.com/opengauss/website/issues/255</v>
       </c>
       <c r="F2">
@@ -829,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -892,7 +897,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1000,7 +1005,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1108,7 +1113,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1216,7 +1221,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1324,13 +1329,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-26 06:08:23</v>
+        <v>2026-07-27 06:18:48</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1369,7 +1374,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-28
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,10 +470,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/188
-https://atomgit.com/openeuler/openEuler-portal/issues/190
-https://atomgit.com/openeuler/openEuler-portal/issues/219
-https://atomgit.com/openeuler/openEuler-portal/issues/191</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/217</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -503,10 +500,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P2">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -569,7 +566,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -677,7 +674,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -785,13 +782,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -799,9 +796,12 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
 https://atomgit.com/opengauss/website/issues/253
+https://atomgit.com/opengauss/website/issues/257
 https://atomgit.com/opengauss/website/issues/254
+https://atomgit.com/opengauss/website/issues/258
+https://atomgit.com/opengauss/website/issues/255
 https://atomgit.com/opengauss/website/issues/266
-https://atomgit.com/opengauss/website/issues/255</v>
+https://atomgit.com/opengauss/website/issues/298</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -828,13 +828,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +897,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1005,7 +1005,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1113,7 +1113,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1221,13 +1221,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1266,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1329,13 +1329,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-27 06:18:48</v>
+        <v>2026-07-28 05:56:50</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1368,13 +1368,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-29
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,21 +456,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/217</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -500,7 +499,7 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -566,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -674,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -782,26 +781,21 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/253
-https://atomgit.com/opengauss/website/issues/257
-https://atomgit.com/opengauss/website/issues/254
-https://atomgit.com/opengauss/website/issues/258
-https://atomgit.com/opengauss/website/issues/255
-https://atomgit.com/opengauss/website/issues/266
-https://atomgit.com/opengauss/website/issues/298</v>
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/303
+https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/304</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -813,7 +807,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -828,13 +822,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P2">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +891,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1005,7 +999,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1113,7 +1107,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1221,13 +1215,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1266,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1329,13 +1323,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-28 05:56:50</v>
+        <v>2026-07-29 06:01:24</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1374,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-30
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,20 +456,23 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187
+https://atomgit.com/openeuler/openEuler-portal/issues/223
+https://atomgit.com/openeuler/openEuler-portal/issues/224
+https://atomgit.com/openeuler/openEuler-portal/issues/225</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -502,7 +505,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -565,7 +568,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +676,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -781,13 +784,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -822,10 +825,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -891,7 +894,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -999,7 +1002,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1107,7 +1110,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1215,7 +1218,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1323,13 +1326,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-29 06:01:24</v>
+        <v>2026-07-30 05:39:41</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1368,7 +1371,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-07-31
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -471,6 +471,7 @@
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/223
+https://atomgit.com/openeuler/openEuler-portal/issues/227
 https://atomgit.com/openeuler/openEuler-portal/issues/224
 https://atomgit.com/openeuler/openEuler-portal/issues/225</v>
       </c>
@@ -568,7 +569,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -676,7 +677,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -782,23 +783,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/303
-https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/304</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/opengauss/website/issues/252</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -810,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -825,10 +824,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -894,7 +893,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1002,7 +1001,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1110,7 +1109,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1218,16 +1217,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
-        <v>成功</v>
+        <v>失败</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>Cannot create property 'border-width' on string 'inherit'</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -1257,7 +1256,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1326,13 +1325,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-30 05:39:41</v>
+        <v>2026-07-31 06:14:09</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1347,13 +1346,13 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I2">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="J2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1365,13 +1364,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-01
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -471,8 +471,9 @@
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/223
+https://atomgit.com/openeuler/openEuler-portal/issues/229
+https://atomgit.com/openeuler/openEuler-portal/issues/224
 https://atomgit.com/openeuler/openEuler-portal/issues/227
-https://atomgit.com/openeuler/openEuler-portal/issues/224
 https://atomgit.com/openeuler/openEuler-portal/issues/225</v>
       </c>
       <c r="F2">
@@ -506,7 +507,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -569,7 +570,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -677,7 +678,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -783,21 +784,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/opengauss/website/issues/252</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/315</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -824,10 +826,10 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -893,7 +895,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1001,7 +1003,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1109,7 +1111,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1217,7 +1219,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1325,7 +1327,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-07-31 06:14:09</v>
+        <v>2026-08-01 06:01:49</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-02
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,25 +456,20 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/223
-https://atomgit.com/openeuler/openEuler-portal/issues/229
-https://atomgit.com/openeuler/openEuler-portal/issues/224
-https://atomgit.com/openeuler/openEuler-portal/issues/227
-https://atomgit.com/openeuler/openEuler-portal/issues/225</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -507,7 +502,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -678,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -786,20 +781,22 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/315</v>
+https://atomgit.com/opengauss/website/issues/316
+https://atomgit.com/opengauss/website/issues/317
+https://atomgit.com/opengauss/website/issues/318</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -826,13 +823,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +892,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1003,7 +1000,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1111,7 +1108,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1219,7 +1216,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1327,13 +1324,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-01 06:01:49</v>
+        <v>2026-08-02 05:55:02</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1366,13 +1363,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-03
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,20 +456,25 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/187
+https://atomgit.com/openeuler/openEuler-portal/issues/230
+https://atomgit.com/openeuler/openEuler-portal/issues/231
+https://atomgit.com/openeuler/openEuler-portal/issues/232
+https://atomgit.com/openeuler/openEuler-portal/issues/233
+https://atomgit.com/openeuler/openEuler-portal/issues/234</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -502,7 +507,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -565,7 +570,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +678,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -779,24 +784,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/316
-https://atomgit.com/opengauss/website/issues/317
-https://atomgit.com/opengauss/website/issues/318</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/opengauss/website/issues/252</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -823,13 +825,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -892,7 +894,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1000,7 +1002,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1108,7 +1110,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1216,7 +1218,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1324,7 +1326,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-02 05:55:02</v>
+        <v>2026-08-03 06:11:34</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1351,7 +1353,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1363,7 +1365,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-04
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,7 +456,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -472,9 +472,9 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/230
 https://atomgit.com/openeuler/openEuler-portal/issues/231
+https://atomgit.com/openeuler/openEuler-portal/issues/234
 https://atomgit.com/openeuler/openEuler-portal/issues/232
-https://atomgit.com/openeuler/openEuler-portal/issues/233
-https://atomgit.com/openeuler/openEuler-portal/issues/234</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/235</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -570,7 +570,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -678,7 +678,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -784,21 +784,24 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/opengauss/website/issues/252</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/321
+https://atomgit.com/opengauss/website/issues/322
+https://atomgit.com/opengauss/website/issues/323</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -828,10 +831,10 @@
         <v>2</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -894,7 +897,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1002,7 +1005,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1110,7 +1113,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1218,7 +1221,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1326,13 +1329,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-03 06:11:34</v>
+        <v>2026-08-04 05:47:30</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1353,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1371,7 +1374,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-05
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>271</v>
+        <v>288</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -472,8 +472,9 @@
 https://atomgit.com/openeuler/openEuler-portal/issues/187
 https://atomgit.com/openeuler/openEuler-portal/issues/230
 https://atomgit.com/openeuler/openEuler-portal/issues/231
+https://atomgit.com/openeuler/openEuler-portal/issues/232
 https://atomgit.com/openeuler/openEuler-portal/issues/234
-https://atomgit.com/openeuler/openEuler-portal/issues/232
+https://atomgit.com/openeuler/openEuler-portal/issues/238
 https://atomgit.com/openeuler/openEuler-portal/issues/235</v>
       </c>
       <c r="F2">
@@ -507,7 +508,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>10</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +571,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -678,7 +679,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -786,21 +787,19 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/321
-https://atomgit.com/opengauss/website/issues/322
 https://atomgit.com/opengauss/website/issues/323</v>
       </c>
       <c r="F2">
@@ -831,10 +830,10 @@
         <v>2</v>
       </c>
       <c r="O2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P2">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +896,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1005,7 +1004,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1113,7 +1112,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1221,7 +1220,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1329,13 +1328,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-04 05:47:30</v>
+        <v>2026-08-05 05:51:39</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1356,7 +1355,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1368,13 +1367,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-06
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,12 +470,9 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/230
 https://atomgit.com/openeuler/openEuler-portal/issues/231
-https://atomgit.com/openeuler/openEuler-portal/issues/232
-https://atomgit.com/openeuler/openEuler-portal/issues/234
-https://atomgit.com/openeuler/openEuler-portal/issues/238
-https://atomgit.com/openeuler/openEuler-portal/issues/235</v>
+https://atomgit.com/openeuler/openEuler-portal/issues/235
+https://atomgit.com/openeuler/openEuler-portal/issues/234</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -508,7 +505,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +568,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -679,7 +676,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -787,20 +784,24 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/323</v>
+https://atomgit.com/opengauss/website/issues/324
+https://atomgit.com/opengauss/website/issues/325
+https://atomgit.com/opengauss/website/issues/326
+https://atomgit.com/opengauss/website/issues/327
+https://atomgit.com/opengauss/website/issues/328</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -827,13 +828,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -896,7 +897,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1004,7 +1005,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1112,7 +1113,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1220,7 +1221,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1328,13 +1329,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-05 05:51:39</v>
+        <v>2026-08-06 05:49:05</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1355,7 +1356,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,13 +1368,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-07
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,26 +454,22 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
-        <v>成功</v>
+        <v>失败</v>
       </c>
       <c r="C2">
-        <v>275</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
+        <v>spawnSync /bin/sh ETIMEDOUT</v>
+      </c>
+      <c r="E2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/187
-https://atomgit.com/openeuler/openEuler-portal/issues/231
-https://atomgit.com/openeuler/openEuler-portal/issues/235
-https://atomgit.com/openeuler/openEuler-portal/issues/234</v>
-      </c>
       <c r="F2">
         <v>0</v>
       </c>
@@ -484,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -499,13 +495,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -568,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -676,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -784,24 +780,24 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/329
 https://atomgit.com/opengauss/website/issues/324
-https://atomgit.com/opengauss/website/issues/325
 https://atomgit.com/opengauss/website/issues/326
 https://atomgit.com/opengauss/website/issues/327
-https://atomgit.com/opengauss/website/issues/328</v>
+https://atomgit.com/opengauss/website/issues/330</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -831,10 +827,10 @@
         <v>3</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +893,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1005,7 +1001,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1113,7 +1109,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1221,7 +1217,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
         <v>失败</v>
@@ -1329,13 +1325,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-06 05:49:05</v>
+        <v>2026-08-07 04:55:35</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1368,13 +1364,13 @@
         <v>0</v>
       </c>
       <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
         <v>3</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-08
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,24 +456,19 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-07 08:54:55</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/231
-https://atomgit.com/openeuler/openEuler-portal/issues/234
-https://atomgit.com/openeuler/openEuler-portal/issues/235
-https://atomgit.com/openeuler/openEuler-portal/issues/241
-https://atomgit.com/openeuler/openEuler-portal/issues/242
 https://atomgit.com/openeuler/openEuler-portal/issues/243</v>
       </c>
       <c r="F2">
@@ -504,10 +499,10 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P2">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +565,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-07 08:54:55</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -678,7 +673,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-07 08:54:55</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -784,24 +779,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-07 08:54:55</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/324
-https://atomgit.com/opengauss/website/issues/326
-https://atomgit.com/opengauss/website/issues/331</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/opengauss/website/issues/252</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -828,13 +820,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +889,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-07 08:54:55</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1005,7 +997,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-07 08:54:55</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1113,7 +1105,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-07 08:54:55</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1223,13 +1215,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-07 12:01:28</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1237,11 +1229,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153
-https://atomgit.com/openUBMC/website/issues/154
-https://atomgit.com/openUBMC/website/issues/155
-https://atomgit.com/openUBMC/website/issues/156
-https://atomgit.com/openUBMC/website/issues/157</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1274,7 +1262,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1335,21 +1323,24 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-07 08:54:55</v>
+        <v>2026-08-08 04:09:10</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v/>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
+https://atomgit.com/hifloat/hifloat-portal/issues/5
+https://atomgit.com/hifloat/hifloat-portal/issues/6
+https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1376,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-09
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,22 +454,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
-https://atomgit.com/openeuler/openEuler-portal/issues/243</v>
+      <c r="E2" t="str">
+        <v>https://atomgit.com/openeuler/openEuler-portal/issues/185</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -499,7 +498,7 @@
         <v>0</v>
       </c>
       <c r="O2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -565,7 +564,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -673,7 +672,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -781,7 +780,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -889,7 +888,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -997,7 +996,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1105,7 +1104,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1215,7 +1214,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1325,13 +1324,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-08 04:09:10</v>
+        <v>2026-08-09 04:21:53</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,7 +1339,8 @@
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
-https://atomgit.com/hifloat/hifloat-portal/issues/7</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1367,7 +1367,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-10
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -454,21 +454,28 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>260</v>
+        <v>297</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/openeuler/openEuler-portal/issues/185</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
+https://atomgit.com/openeuler/openEuler-portal/issues/249
+https://atomgit.com/openeuler/openEuler-portal/issues/250
+https://atomgit.com/openeuler/openEuler-portal/issues/251
+https://atomgit.com/openeuler/openEuler-portal/issues/252
+https://atomgit.com/openeuler/openEuler-portal/issues/253
+https://atomgit.com/openeuler/openEuler-portal/issues/254
+https://atomgit.com/openeuler/openEuler-portal/issues/255</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -501,7 +508,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -564,7 +571,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -672,7 +679,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -778,21 +785,23 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str">
-        <v>https://atomgit.com/opengauss/website/issues/252</v>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
+https://atomgit.com/opengauss/website/issues/333
+https://atomgit.com/opengauss/website/issues/334</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -819,13 +828,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -888,7 +897,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -996,7 +1005,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1104,7 +1113,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1214,13 +1223,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1228,7 +1237,11 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153</v>
+https://atomgit.com/openUBMC/website/issues/153
+https://atomgit.com/openUBMC/website/issues/154
+https://atomgit.com/openUBMC/website/issues/155
+https://atomgit.com/openUBMC/website/issues/156
+https://atomgit.com/openUBMC/website/issues/158</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1261,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1324,13 +1337,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-09 04:21:53</v>
+        <v>2026-08-10 04:42:46</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1340,7 +1353,10 @@
 https://atomgit.com/hifloat/hifloat-portal/issues/5
 https://atomgit.com/hifloat/hifloat-portal/issues/6
 https://atomgit.com/hifloat/hifloat-portal/issues/7
-https://atomgit.com/hifloat/hifloat-portal/issues/8</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/10
+https://atomgit.com/hifloat/hifloat-portal/issues/11
+https://atomgit.com/hifloat/hifloat-portal/issues/12
+https://atomgit.com/hifloat/hifloat-portal/issues/13</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1355,7 +1371,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1367,13 +1383,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: 更新 daily check 历史 2026-08-11
</commit_message>
<xml_diff>
--- a/daily-check-history.xlsx
+++ b/daily-check-history.xlsx
@@ -456,13 +456,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -470,11 +470,9 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openeuler/openEuler-portal/issues/185
 https://atomgit.com/openeuler/openEuler-portal/issues/249
-https://atomgit.com/openeuler/openEuler-portal/issues/250
+https://atomgit.com/openeuler/openEuler-portal/issues/252
+https://atomgit.com/openeuler/openEuler-portal/issues/254
 https://atomgit.com/openeuler/openEuler-portal/issues/251
-https://atomgit.com/openeuler/openEuler-portal/issues/252
-https://atomgit.com/openeuler/openEuler-portal/issues/253
-https://atomgit.com/openeuler/openEuler-portal/issues/254
 https://atomgit.com/openeuler/openEuler-portal/issues/255</v>
       </c>
       <c r="F2">
@@ -508,7 +506,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +569,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -679,7 +677,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -785,23 +783,21 @@
         <v>tdk-schema-semantic</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
         <v/>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">https://atomgit.com/opengauss/website/issues/252
-https://atomgit.com/opengauss/website/issues/333
-https://atomgit.com/opengauss/website/issues/334</v>
+      <c r="E2" t="str">
+        <v/>
       </c>
       <c r="F2">
         <v>0</v>
@@ -828,13 +824,13 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +893,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1005,7 +1001,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>跳过</v>
@@ -1113,7 +1109,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1223,13 +1219,13 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
       </c>
       <c r="C2">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -1237,11 +1233,7 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/openUBMC/website/issues/151
 https://atomgit.com/openUBMC/website/issues/152
-https://atomgit.com/openUBMC/website/issues/153
-https://atomgit.com/openUBMC/website/issues/154
-https://atomgit.com/openUBMC/website/issues/155
-https://atomgit.com/openUBMC/website/issues/156
-https://atomgit.com/openUBMC/website/issues/158</v>
+https://atomgit.com/openUBMC/website/issues/153</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1274,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1337,7 +1329,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-08-10 04:42:46</v>
+        <v>2026-08-11 04:29:32</v>
       </c>
       <c r="B2" t="str">
         <v>成功</v>
@@ -1351,12 +1343,12 @@
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">https://atomgit.com/hifloat/hifloat-portal/issues/4
 https://atomgit.com/hifloat/hifloat-portal/issues/5
-https://atomgit.com/hifloat/hifloat-portal/issues/6
 https://atomgit.com/hifloat/hifloat-portal/issues/7
+https://atomgit.com/hifloat/hifloat-portal/issues/8
 https://atomgit.com/hifloat/hifloat-portal/issues/10
-https://atomgit.com/hifloat/hifloat-portal/issues/11
 https://atomgit.com/hifloat/hifloat-portal/issues/12
-https://atomgit.com/hifloat/hifloat-portal/issues/13</v>
+https://atomgit.com/hifloat/hifloat-portal/issues/13
+https://atomgit.com/hifloat/hifloat-portal/issues/11</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1371,7 +1363,7 @@
         <v>36</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -1383,7 +1375,7 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>0</v>

</xml_diff>